<commit_message>
feat: add bidirectional requirement traceability validator and deduplication check
</commit_message>
<xml_diff>
--- a/templates/testcase-template.xlsx
+++ b/templates/testcase-template.xlsx
@@ -1037,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1114,10 +1114,58 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
+          <t>Tỷ lệ Truy vết Yêu cầu (Traceability Rate):</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>100% (3/3 yêu cầu trọng yếu đã có test case bao phủ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Yêu cầu Trọng yếu Chưa có Test Case (Orphan):</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Không có (0) - Đạt chuẩn 100% bao phủ nghiệp vụ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Test Case Ảo Không có Căn cứ Code/Spec:</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Không có (0) - 100% test case có mã đối soát thực tế</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Test Case Trùng lặp Mục tiêu (Duplicates):</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Không có (0) - Bộ test case độc lập và tối giản</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
           <t>Các Luồng Nghiệp vụ Đã Bao Phủ:</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>• Luồng Đăng nhập hợp lệ chính thống (Happy Path)
 • Cơ chế phòng thủ chống spam click submit liên tục (useSubmitOnce)
@@ -1125,26 +1173,26 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Vùng Rủi ro Chưa Bao Phủ / Tồn đọng:</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>• Luồng xác thực đăng nhập một lần (SSO OAuth2 qua Google/Microsoft)
 • Luồng mở khoá bằng mã PIN vật lý bảo mật phần cứng</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Giả định Môi trường &amp; Dữ liệu:</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>• Môi trường Staging không bật Google reCAPTCHA v3
 • Database có sẵn tài khoản mẫu đã kích hoạt và không bị khoá</t>

</xml_diff>

<commit_message>
feat: enforce non-IT accessible business terminology standard for test cases without reducing test quotas
</commit_message>
<xml_diff>
--- a/templates/testcase-template.xlsx
+++ b/templates/testcase-template.xlsx
@@ -693,14 +693,14 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1. Mở trang /dang-nhap
-2. Nhập username và password
-3. Bấm Đăng nhập</t>
+          <t>1. Mở màn hình Đăng nhập (/dang-nhap)
+2. Nhập tên đăng nhập và mật khẩu hợp lệ
+3. Bấm nút 'Đăng nhập'</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Hệ thống xác thực thành công và điều hướng vào Dashboard</t>
+          <t>Hệ thống xác thực thành công, màn hình tự động chuyển hướng vào Trang chủ Dashboard</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -743,28 +743,30 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Chống spam click nút Đăng nhập khi mạng lag</t>
+          <t>Kiểm tra giới hạn số lần gửi: Chặn gửi liên tục khi tài khoản yêu cầu quá giới hạn 3 lần trong 24 giờ</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Nhập đúng thông tin tài khoản</t>
+          <t>Tài khoản nhân viên đã gửi 3 yêu cầu cấp lại trong 24 giờ qua</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Tên đăng nhập: user01, Mật khẩu: Pass@123</t>
+          <t>Mã nhân viên: NV-102 (đã đạt giới hạn 3 lần/24h)</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>1. Nhập thông tin đăng nhập
-2. Bấm liên tiếp 3 lần nút Đăng nhập trong 500ms</t>
+          <t>1. Mở màn hình Quên Mật Khẩu
+2. Nhập Mã nhân viên NV-102 vào ô nhập liệu
+3. Bấm nút 'Gửi Yêu Cầu' lần thứ 4</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Nút chuyển trạng thái loading, vô hiệu hoá click trùng, chỉ gửi 1 request API duy nhất</t>
+          <t>- Trên màn hình: Hiển thị thông báo thành công chung (Mã: VBO-QM-03) nhằm bảo mật an toàn tài khoản.
+- Trong hệ thống: Không phát sinh thêm bản ghi yêu cầu mới do đã vượt quá 3 lần/24h.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -780,12 +782,12 @@
       <c r="J3" s="8" t="inlineStr"/>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>SPEC-HT-26 (useSubmitOnce)</t>
+          <t>SPEC-HT-26 (RateLimiting)</t>
         </is>
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>Bảo vệ chống nhảy bộ đếm sai khoá tài khoản oan</t>
+          <t>Bảo vệ chống spam liên tục và tránh lộ trạng thái tài khoản</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
@@ -807,28 +809,28 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Chuyển đổi Tab định danh (Mã NV -&gt; SĐT) tự động xoá ô nhập</t>
+          <t>Chuyển đổi hình thức đăng nhập (Mã nhân viên sang Số điện thoại) tự động xoá ô nhập liệu</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Đang ở màn hình đăng nhập mặc định Tab Mã NV</t>
+          <t>Đang ở màn hình đăng nhập mặc định chọn tab Mã nhân viên</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Chuỗi gõ dở dang: NV009988</t>
+          <t>Dữ liệu gõ dở dang: NV009988</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>1. Gõ chuỗi 'NV009988' vào ô Mã NV
-2. Bấm đổi sang Tab 'Số điện thoại'</t>
+          <t>1. Nhập 'NV009988' vào ô Mã nhân viên
+2. Bấm chọn tab 'Số điện thoại'</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Giao diện chuyển sang Tab SĐT, ô định danh bị xoá trắng chuỗi cũ, placeholder đổi sang dạng SĐT</t>
+          <t>Giao diện chuyển sang tab Số điện thoại, ô nhập liệu tự động được xoá trắng nội dung cũ, gợi ý đổi sang định dạng Số điện thoại</t>
         </is>
       </c>
       <c r="H4" s="10" t="inlineStr">

</xml_diff>

<commit_message>
fix(excel): implement dynamic row height auto-scale, 85% opening zoom, and vertical top alignment
</commit_message>
<xml_diff>
--- a/templates/testcase-template.xlsx
+++ b/templates/testcase-template.xlsx
@@ -180,31 +180,31 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -213,7 +213,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="left" vertical="top" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -578,24 +578,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -665,7 +665,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="92" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>TC-AUTH-001</t>
@@ -730,7 +730,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1">
+    <row r="3" ht="124" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>TC-AUTH-002</t>
@@ -796,7 +796,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1">
+    <row r="4" ht="92" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>TC-AUTH-003</t>
@@ -874,6 +874,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -881,19 +882,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -938,7 +939,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>GAP-001</t>
@@ -980,7 +981,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>GAP-002</t>
@@ -1030,6 +1031,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -1042,8 +1044,8 @@
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -1053,7 +1055,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Tên Phân hệ / Module:</t>
@@ -1065,7 +1067,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Tổng số Test Cases Thiết kế:</t>
@@ -1073,11 +1075,11 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>3 (Mẫu - Tiêu chuẩn thực tế: 7–10 Chặn, 5–7 Sai)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>3 ca mẫu (Phân bổ theo Risk-Based Coverage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Số ca Sẵn sàng Tự động hoá (Yes):</t>
@@ -1089,7 +1091,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Số ca Yêu cầu Kiểm thử Thủ công (No):</t>
@@ -1101,7 +1103,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Phân bổ Mức độ Nghiêm trọng:</t>
@@ -1113,7 +1115,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Tỷ lệ Truy vết Yêu cầu (Traceability Rate):</t>
@@ -1125,7 +1127,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Yêu cầu Trọng yếu Chưa có Test Case (Orphan):</t>
@@ -1137,7 +1139,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Test Case Ảo Không có Căn cứ Code/Spec:</t>
@@ -1149,7 +1151,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Test Case Trùng lặp Mục tiêu (Duplicates):</t>
@@ -1161,7 +1163,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="74" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Các Luồng Nghiệp vụ Đã Bao Phủ:</t>
@@ -1175,7 +1177,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="58" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Vùng Rủi ro Chưa Bao Phủ / Tồn đọng:</t>
@@ -1188,7 +1190,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Giả định Môi trường &amp; Dữ liệu:</t>

</xml_diff>